<commit_message>
refactor: freeze trajectory v3 review release
</commit_message>
<xml_diff>
--- a/test/客服/输入附件-扩展版.xlsx
+++ b/test/客服/输入附件-扩展版.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complaints" sheetId="1" r:id="R0256d3da388b42a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="responses" sheetId="2" r:id="R3c2fedd35e1e49c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complaints" sheetId="1" r:id="R139523e82d1c4b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="responses" sheetId="2" r:id="Rd2441c9a0857499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="narratives" sheetId="3" r:id="R8cbcf559338d48fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +54,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -65,11 +66,45 @@
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -820,6 +855,7 @@
     <ns0:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
     <ns0:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
     <ns0:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <ns0:col min="5" max="5" width="65" hidden="0" customWidth="1"/>
   </ns0:cols>
   <ns0:sheetData>
     <ns0:row r="1" ht="15" hidden="0" customHeight="1">
@@ -835,6 +871,422 @@
       <ns0:c r="D1" s="4" t="str">
         <ns0:v>company_response</ns0:v>
       </ns0:c>
+      <ns0:c r="E1" s="5" t="str">
+        <ns0:v>company_public_response</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+      <ns0:c r="A2" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999454</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T23:00:25.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T23:10:13.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E2" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Company has responded to the consumer and the CFPB and chooses not to provide a public response</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
+      <ns0:c r="A3" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9998304</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T01:00:19.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T01:00:22.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D3" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E3" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Company has responded to the consumer and the CFPB and chooses not to provide a public response</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A4" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9998965</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T23:55:08.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:08:22.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D4" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E4" s="6"/>
+    </ns0:row>
+    <ns0:row r="5" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A5" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9717197</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-08-05T10:19:29.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-08-05T10:19:31.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E5" s="6"/>
+    </ns0:row>
+    <ns0:row r="6" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A6" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999759</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T17:27:34.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T17:34:17.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E6" s="6"/>
+    </ns0:row>
+    <ns0:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <ns0:c r="A7" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999984</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T21:46:19.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T21:46:27.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Company has responded to the consumer and the CFPB and chooses not to provide a public response</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A8" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9998629</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:31:41.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:32:00.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" s="6"/>
+    </ns0:row>
+    <ns0:row r="9" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A9" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9777751</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-08-12T01:13:42.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-08-12T01:26:08.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" s="6"/>
+    </ns0:row>
+    <ns0:row r="10" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A10" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999727</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T17:24:21.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T17:27:11.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D10" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E10" s="6"/>
+    </ns0:row>
+    <ns0:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <ns0:c r="A11" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999064</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:58:39.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:59:00.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D11" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Company has responded to the consumer and the CFPB and chooses not to provide a public response</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A12" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999591</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T18:23:57.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T18:24:00.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D12" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E12" s="6"/>
+    </ns0:row>
+    <ns0:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <ns0:c r="A13" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9997644</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T02:24:37.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T02:30:52.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D13" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E13" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Company has responded to the consumer and the CFPB and chooses not to provide a public response</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A14" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9998761</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:05:09.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C14" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-04T00:05:25.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D14" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E14" s="6"/>
+    </ns0:row>
+    <ns0:row r="15" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A15" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9996794</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T19:29:17.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C15" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T19:29:35.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D15" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E15" s="6"/>
+    </ns0:row>
+    <ns0:row r="16" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A16" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9899292</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-08-23T19:19:57.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-08-23T19:47:00.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D16" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E16" s="6"/>
+    </ns0:row>
+    <ns0:row r="17" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A17" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">9999710</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T17:20:12.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2024-09-03T17:20:15.000Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E17" s="6"/>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <ns0:col min="2" max="2" width="65" hidden="0" customWidth="1"/>
+    <ns0:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="A1" s="4" t="str">
+        <ns0:v>complaint_id</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" s="5" t="str">
+        <ns0:v>narrative_excerpt</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" s="11" t="str">
+        <ns0:v>excerpt_truncated</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="2" ht="15" hidden="0" customHeight="1">
       <ns0:c r="A2" s="2" t="inlineStr">
@@ -842,42 +1294,29 @@
           <ns0:t xml:space="preserve">9999454</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B2" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T23:00:25.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C2" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T23:10:13.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D2" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B2" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3" ht="211.1999969482422" hidden="0" customHeight="1">
       <ns0:c r="A3" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9998304</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T01:00:19.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T01:00:22.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
+      <ns0:c r="B3" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">XXXX XXXX XXXX XXXX XXXX XXXX XXXX XXXX, TX XXXX Consumer Financial Protection Bureau XXXX XXXX XXXX XXXX  XXXX, IA XXXX Subject : Formal Complaint Regarding Inaccurate Late Payment Information on Credit Report Dear CFPB, I am writing to formally lodge a complaint regarding inaccurate late payment information reported by XXXX CARDS on my credit report. The late payments in question were marked on the following account ( XXXX ) on the respective date ( XXXX ) : LATE PAYMENT DAY : XX/XX/XXXX LATE PAYMENT DAY : XX/XX/XXXX LATE PAYMENT DAY : XX/XX/XXXX LATE PAYMENT DAY : XX/XX/XXXX LATE PAYMENT DAY : XX/XX/XXXX LATE PAYMENT DAY : XX/XX/XXXX Under 15 USC 1681 ( a ) ( 2 ) ( A ) ( i ), it is my understanding that my consumer report should not contain information related solely to transactions or experiences between myself, the consumer, and the person or entity providing the report. The inclusion of late payments as part of my payment history negatively impacts my consumer report, and I believe this is in direct violation of the aforementioned statute. 
+Additionally, I am requesting that XXXX CARDS provide, in writing, the reasonable procedures it has adopted to ensure that each periodic </ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" s="9" t="b">
+        <ns0:v>1</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="4" ht="15" hidden="0" customHeight="1">
@@ -886,42 +1325,31 @@
           <ns0:t xml:space="preserve">9998965</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B4" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T23:55:08.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C4" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:08:22.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D4" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B4" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" ht="237.60000610351562" hidden="0" customHeight="1">
       <ns0:c r="A5" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9717197</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B5" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-08-05T10:19:29.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C5" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-08-05T10:19:31.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D5" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
+      <ns0:c r="B5" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I am writing to formally notify you of serious violations concerning the furnishing of consumer data that has come to my attention. As a secondary consumer reporting agency, you are required to adhere strictly to federal and state laws governing consumer credit and reporting practices. Your recent actions have violated these laws, specifically the Fair Debt Collection Practices Act ( FDCPA ), 15 U.S.C. 1692c ( c ), and relevant case law, including XXXXXXXX XXXX XXXX XXXX XXXXXXXX, XXXX XXXX. XXXX. 
+Under the FDCPA, any consumer reporting agency must refrain from disclosing information to third parties without proper consent, especially when such information is inaccurate or unverifiable. In this instance, your agency has furnished data that does not comply with these legal standards. 
+Furthermore, the case of XXXX XXXX XXXX XXXX XXXX illustrates the consequences of failing to uphold these standards, highlighting the judicial recognition of consumers ' rights to accurate credit reporting. Your actions not only contravene established case law but also expose you to significant legal liabilities. 
+According to the FDCPA, consumers may seek damages for violations, including statutor</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" s="9" t="b">
+        <ns0:v>1</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="6" ht="15" hidden="0" customHeight="1">
@@ -930,20 +1358,13 @@
           <ns0:t xml:space="preserve">9999759</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T17:27:34.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T17:34:17.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
+      <ns0:c r="B6" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" s="9" t="b">
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="7" ht="15" hidden="0" customHeight="1">
@@ -952,86 +1373,61 @@
           <ns0:t xml:space="preserve">9999984</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T21:46:19.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T21:46:27.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B7" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8" ht="79.19999694824219" hidden="0" customHeight="1">
       <ns0:c r="A8" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9998629</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B8" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:31:41.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C8" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:32:00.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D8" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B8" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I AM WRITING TO DELETE THE FOLLOWING INFORMATION FROM MY FILE.THE ITEMS I WANT DELETED ARE LISTED IN THE REPORT. I AM A VICTIM OF IDENTITY THEFT AND I DID NOT MAKE THE CHARGE.I REPORTED THE THEFT TO THE FEDERAL TRADE COMMISSION AND I ALSO HAVE ENCLOSED COPIES TO THE FEDERAL TRADE COMMISSION IDENTITY THEFT AFFIDAVIT.PLEASE DELETE THESE ITEMS AS AS SOON AS POSSIBLE.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9" ht="250.8000030517578" hidden="0" customHeight="1">
       <ns0:c r="A9" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9777751</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B9" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-08-12T01:13:42.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C9" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-08-12T01:26:08.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D9" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B9" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">On XX/XX/year&gt;, I discovered that an unauthorized transaction of {$8000.00} was processed on my account ( Account XXXX : XXXX ). This transaction occurred while my virtual credit card was locked, which should have prevented any such activity from being processed. I did not authorize or approve this transaction. 
+Upon discovering the unauthorized transaction, I immediately contacted my bank, Current Bank, and spoke with a customer service representative named XXXX. During this conversation, I initiated a dispute for the transaction under dispute number XXXX. As of XXXX XXXX  on XX/XX/year&gt;, my account reflects that this transaction is under dispute. 
+Despite my clear request to restore my account balance to the state it was in before this unauthorized transaction, XXXX was unable to provide a satisfactory explanation for why my account balance had not been corrected. 
+I believe that the banks actions may be in violation of Regulation Z under the Truth in Lending Act ( XXXX XXXX XXXX ), which prohibits a creditor from taking action to collect on any disputed portion of a transaction or from deducting disputed amounts and related charges from a consumers credit limit while the disp</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" s="9" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10" ht="105.5999984741211" hidden="0" customHeight="1">
       <ns0:c r="A10" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9999727</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B10" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T17:24:21.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C10" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T17:27:11.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D10" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
+      <ns0:c r="B10" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">In the quiet humdrum of everyday life, a sudden jolt shattered the tranquility : I had become a victim of identity theft. Like a thief in the night, unseen hands had stolen my personal information, plunging me into a bewildering maze of uncertainty. With each fraudulent transaction and unauthorized account, the breach of trust cut deep, leaving me grappling with the unsettling reality of a violated identity. Yet, in the midst of chaos, a glimmer of resilience emerged, a resolve to reclaim what was rightfully mine and restore the harmony stolen by unseen adversaries. These are the following accounts need to be removed :</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" s="9" t="b">
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1040,20 +1436,13 @@
           <ns0:t xml:space="preserve">9999064</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B11" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:58:39.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C11" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:59:00.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D11" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
+      <ns0:c r="B11" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" s="9" t="b">
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1062,108 +1451,81 @@
           <ns0:t xml:space="preserve">9999591</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B12" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T18:23:57.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C12" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T18:24:00.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D12" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B12" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13" ht="52.79999923706055" hidden="0" customHeight="1">
       <ns0:c r="A13" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9997644</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B13" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T02:24:37.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C13" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T02:30:52.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D13" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B13" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I'm really not sure what happened. I have mailed off letters to the credit bureaus continuously and thus far I have not gotten a response. My name is XXXX XXXX XXXX and I am filing this complaint for falsely reporting misleading information. There is no third party involved. Please review the uploaded letters.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14" ht="264" hidden="0" customHeight="1">
       <ns0:c r="A14" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9998761</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:05:09.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-04T00:05:25.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B14" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I am writing to formally request validation of the debt referenced above. As the account in question is being reported as a collection account on my credit report, I am exercising my rights under the Fair Debt Collection Practices Act ( FDCPA ) to request verification of this debt. 
+Please provide me with the following information : 1. The original creditors name and address. 
+2. A complete account history, including any charges, payments, or fees that have been added to the account. 
+3. Proof that you are legally entitled to collect on this debt, including a copy of the assignment contract or any agreement transferring the debt to your agency. 
+4. A copy of the original signed contract or agreement that created this debt. 
+5. Verification of the amount claimed, including any interest, fees, or other charges that have been added to the balance. 
+According to my records, the details of the account are as follows : Account Name : XXXX XXXX XXXX 
+Account Number : XXXX Account Type : Collection Date Opened : XX/XX/XXXX Status : Collection account, {$6000.00} past due as of XX/XX/XXXX Balance : {$6000.00} Please be advised that you are required to provide this information within 30 da</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C14" s="9" t="b">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15" ht="92.4000015258789" hidden="0" customHeight="1">
       <ns0:c r="A15" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9996794</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B15" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T19:29:17.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C15" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T19:29:35.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D15" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16" ht="15" hidden="0" customHeight="1">
+      <ns0:c r="B15" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">This account was charged off on the following date : XXXXXXX Since then the account has repeatedly been updated as charged off every month. This is an update in the payment history. A charged off account shouldn't include an active payment history. This inaccurate information falsely manipulates the statute of limitation. Please investigate this account property after I asked you to do it TWICE and your neglect has violated my rights, I am demanding a deletion of the following account : Accounts autombile : Account Number XXXX</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C15" s="9" t="b">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16" ht="211.1999969482422" hidden="0" customHeight="1">
       <ns0:c r="A16" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">9899292</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-08-23T19:19:57.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-08-23T19:47:00.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with explanation</ns0:t>
-        </ns0:is>
+      <ns0:c r="B16" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Dear Sir/Madam, I am contacting you today to file a complaint against First Advantage Corporation located at XXXX XXXX XXXX XXXX XXXX XXXX XXXX, XXXX, GA XXXX. As of today I have submitted three disputes pertaining to the same inaccurate information that they have been reporting to potential employers regarding a felony charge on my criminal record. The XXXXXXXX charge they are referencing was disposed of in the XXXXXXXX XXXX XXXXXXXX XXXX XXXX XXXX on XX/XX/XXXX. The XXXX was reduced to XXXX I sent them all court paperwork to verify this and contact information to the clerk of the court in the correct court system for verification. Because of the information being reported and also the fact that it has been over 90 days since submitting the original information to the company, and more than 60 days since my first dispute, I have lost or been denied employment by several companies which has had a substantial impact on my familys well being. 
+# # # # THE ISSUE # # # # XXXX - They have created a synthetic record : They took an order that they found with reference XXXX XXXX  which was the outcome of a motion to appeal hearing and are mistakenly associating that same reference # with </ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" s="9" t="b">
+        <ns0:v>1</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1172,20 +1534,13 @@
           <ns0:t xml:space="preserve">9999710</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B17" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T17:20:12.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C17" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2024-09-03T17:20:15.000Z</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D17" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Closed with non-monetary relief</ns0:t>
-        </ns0:is>
+      <ns0:c r="B17" s="6" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" s="9" t="b">
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>

</xml_diff>